<commit_message>
continue and finishing (hopefully) the new experiment for prompt with explanation.
</commit_message>
<xml_diff>
--- a/Backup_ToDelete/Aug25Experiments_3_judged_pilot_answers_tagged_WITH_explanation_prompt.xlsx
+++ b/Backup_ToDelete/Aug25Experiments_3_judged_pilot_answers_tagged_WITH_explanation_prompt.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AS31"/>
+  <dimension ref="A1:AV31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -654,10 +654,25 @@
           <t>DeepSeek-V3 Tag for llama-3.1-70b-versatile Answer</t>
         </is>
       </c>
+      <c r="AT1" s="1" t="inlineStr">
+        <is>
+          <t>GPT-4.1-mini Tag for GPT-4-o-mini Answer</t>
+        </is>
+      </c>
+      <c r="AU1" s="1" t="inlineStr">
+        <is>
+          <t>GPT-4.1-mini Tag for Gemini-1.5-flash Answer</t>
+        </is>
+      </c>
+      <c r="AV1" s="1" t="inlineStr">
+        <is>
+          <t>GPT-4.1-mini Tag for llama-3.1-70b-versatile Answer</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B2" t="n">
         <v>2</v>
@@ -672,25 +687,25 @@
         <v>2</v>
       </c>
       <c r="F2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G2" t="n">
         <v>2</v>
       </c>
       <c r="H2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K2" t="n">
         <v>2</v>
       </c>
       <c r="L2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M2" t="n">
         <v>2</v>
@@ -726,7 +741,7 @@
         <v>3</v>
       </c>
       <c r="X2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Y2" t="n">
         <v>3</v>
@@ -735,7 +750,7 @@
         <v>3</v>
       </c>
       <c r="AA2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AB2" t="n">
         <v>2</v>
@@ -750,16 +765,16 @@
         <v>2</v>
       </c>
       <c r="AF2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH2" t="n">
         <v>2</v>
       </c>
       <c r="AI2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AJ2" t="n">
         <v>2</v>
@@ -771,7 +786,7 @@
         <v>2</v>
       </c>
       <c r="AM2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AN2" t="n">
         <v>2</v>
@@ -790,6 +805,15 @@
       </c>
       <c r="AS2" t="n">
         <v>2</v>
+      </c>
+      <c r="AT2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV2" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="3">
@@ -818,16 +842,16 @@
         <v>2</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J3" t="n">
         <v>1</v>
       </c>
       <c r="K3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M3" t="n">
         <v>1</v>
@@ -926,6 +950,15 @@
         <v>2</v>
       </c>
       <c r="AS3" t="n">
+        <v>2</v>
+      </c>
+      <c r="AT3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU3" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV3" t="n">
         <v>2</v>
       </c>
     </row>
@@ -943,13 +976,13 @@
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F4" t="n">
         <v>2</v>
       </c>
       <c r="G4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H4" t="n">
         <v>1</v>
@@ -976,7 +1009,7 @@
         <v>2</v>
       </c>
       <c r="P4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q4" t="n">
         <v>2</v>
@@ -997,10 +1030,10 @@
         <v>2</v>
       </c>
       <c r="W4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="X4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Y4" t="n">
         <v>3</v>
@@ -1015,7 +1048,7 @@
         <v>2</v>
       </c>
       <c r="AC4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AD4" t="n">
         <v>2</v>
@@ -1024,7 +1057,7 @@
         <v>2</v>
       </c>
       <c r="AF4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AG4" t="n">
         <v>2</v>
@@ -1064,6 +1097,15 @@
       </c>
       <c r="AS4" t="n">
         <v>2</v>
+      </c>
+      <c r="AT4" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU4" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV4" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="5">
@@ -1077,7 +1119,7 @@
         <v>2</v>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E5" t="n">
         <v>3</v>
@@ -1086,7 +1128,7 @@
         <v>2</v>
       </c>
       <c r="G5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H5" t="n">
         <v>3</v>
@@ -1101,7 +1143,7 @@
         <v>3</v>
       </c>
       <c r="L5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M5" t="n">
         <v>2</v>
@@ -1137,10 +1179,10 @@
         <v>3</v>
       </c>
       <c r="X5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Y5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Z5" t="n">
         <v>3</v>
@@ -1149,7 +1191,7 @@
         <v>2</v>
       </c>
       <c r="AB5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AC5" t="n">
         <v>3</v>
@@ -1200,6 +1242,15 @@
         <v>3</v>
       </c>
       <c r="AS5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AT5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU5" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV5" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1214,7 +1265,7 @@
         <v>1</v>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E6" t="n">
         <v>2</v>
@@ -1262,13 +1313,13 @@
         <v>1</v>
       </c>
       <c r="T6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U6" t="n">
         <v>1</v>
       </c>
       <c r="V6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W6" t="n">
         <v>2</v>
@@ -1298,7 +1349,7 @@
         <v>1</v>
       </c>
       <c r="AF6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AG6" t="n">
         <v>1</v>
@@ -1307,7 +1358,7 @@
         <v>2</v>
       </c>
       <c r="AI6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AJ6" t="n">
         <v>2</v>
@@ -1316,7 +1367,7 @@
         <v>1</v>
       </c>
       <c r="AL6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AM6" t="n">
         <v>1</v>
@@ -1331,12 +1382,21 @@
         <v>1</v>
       </c>
       <c r="AQ6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AR6" t="n">
         <v>2</v>
       </c>
       <c r="AS6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU6" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV6" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1348,7 +1408,7 @@
         <v>3</v>
       </c>
       <c r="C7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D7" t="n">
         <v>1</v>
@@ -1357,7 +1417,7 @@
         <v>3</v>
       </c>
       <c r="F7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G7" t="n">
         <v>1</v>
@@ -1387,7 +1447,7 @@
         <v>1</v>
       </c>
       <c r="P7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q7" t="n">
         <v>3</v>
@@ -1414,13 +1474,13 @@
         <v>1</v>
       </c>
       <c r="Y7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Z7" t="n">
         <v>3</v>
       </c>
       <c r="AA7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AB7" t="n">
         <v>1</v>
@@ -1432,13 +1492,13 @@
         <v>1</v>
       </c>
       <c r="AE7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AF7" t="n">
         <v>3</v>
       </c>
       <c r="AG7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AH7" t="n">
         <v>2</v>
@@ -1468,18 +1528,27 @@
         <v>2</v>
       </c>
       <c r="AQ7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AR7" t="n">
         <v>3</v>
       </c>
       <c r="AS7" t="n">
+        <v>2</v>
+      </c>
+      <c r="AT7" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU7" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV7" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B8" t="n">
         <v>2</v>
@@ -1488,7 +1557,7 @@
         <v>2</v>
       </c>
       <c r="D8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E8" t="n">
         <v>2</v>
@@ -1506,7 +1575,7 @@
         <v>2</v>
       </c>
       <c r="J8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K8" t="n">
         <v>2</v>
@@ -1524,7 +1593,7 @@
         <v>1</v>
       </c>
       <c r="P8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q8" t="n">
         <v>2</v>
@@ -1545,13 +1614,13 @@
         <v>1</v>
       </c>
       <c r="W8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="X8" t="n">
         <v>2</v>
       </c>
       <c r="Y8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Z8" t="n">
         <v>3</v>
@@ -1572,10 +1641,10 @@
         <v>1</v>
       </c>
       <c r="AF8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AH8" t="n">
         <v>2</v>
@@ -1611,6 +1680,15 @@
         <v>2</v>
       </c>
       <c r="AS8" t="n">
+        <v>2</v>
+      </c>
+      <c r="AT8" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU8" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV8" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1634,7 +1712,7 @@
         <v>3</v>
       </c>
       <c r="G9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H9" t="n">
         <v>3</v>
@@ -1688,13 +1766,13 @@
         <v>3</v>
       </c>
       <c r="Y9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Z9" t="n">
         <v>3</v>
       </c>
       <c r="AA9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AB9" t="n">
         <v>2</v>
@@ -1748,6 +1826,15 @@
         <v>3</v>
       </c>
       <c r="AS9" t="n">
+        <v>3</v>
+      </c>
+      <c r="AT9" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU9" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV9" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1822,7 +1909,7 @@
         <v>3</v>
       </c>
       <c r="X10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Y10" t="n">
         <v>3</v>
@@ -1885,6 +1972,15 @@
         <v>3</v>
       </c>
       <c r="AS10" t="n">
+        <v>2</v>
+      </c>
+      <c r="AT10" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU10" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV10" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1896,10 +1992,10 @@
         <v>3</v>
       </c>
       <c r="C11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E11" t="n">
         <v>3</v>
@@ -1908,16 +2004,16 @@
         <v>1</v>
       </c>
       <c r="G11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H11" t="n">
         <v>2</v>
       </c>
       <c r="I11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K11" t="n">
         <v>2</v>
@@ -1935,7 +2031,7 @@
         <v>1</v>
       </c>
       <c r="P11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q11" t="n">
         <v>3</v>
@@ -1953,7 +2049,7 @@
         <v>1</v>
       </c>
       <c r="V11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W11" t="n">
         <v>2</v>
@@ -1965,13 +2061,13 @@
         <v>3</v>
       </c>
       <c r="Z11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AA11" t="n">
         <v>1</v>
       </c>
       <c r="AB11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AC11" t="n">
         <v>3</v>
@@ -1983,13 +2079,13 @@
         <v>1</v>
       </c>
       <c r="AF11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG11" t="n">
         <v>1</v>
       </c>
       <c r="AH11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AI11" t="n">
         <v>3</v>
@@ -2016,12 +2112,21 @@
         <v>1</v>
       </c>
       <c r="AQ11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AR11" t="n">
         <v>2</v>
       </c>
       <c r="AS11" t="n">
+        <v>2</v>
+      </c>
+      <c r="AT11" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU11" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2051,7 +2156,7 @@
         <v>2</v>
       </c>
       <c r="I12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J12" t="n">
         <v>1</v>
@@ -2075,10 +2180,10 @@
         <v>3</v>
       </c>
       <c r="Q12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S12" t="n">
         <v>1</v>
@@ -2087,7 +2192,7 @@
         <v>2</v>
       </c>
       <c r="U12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V12" t="n">
         <v>2</v>
@@ -2102,10 +2207,10 @@
         <v>3</v>
       </c>
       <c r="Z12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AA12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AB12" t="n">
         <v>3</v>
@@ -2123,7 +2228,7 @@
         <v>3</v>
       </c>
       <c r="AG12" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AH12" t="n">
         <v>2</v>
@@ -2159,6 +2264,15 @@
         <v>2</v>
       </c>
       <c r="AS12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT12" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU12" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV12" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2182,7 +2296,7 @@
         <v>3</v>
       </c>
       <c r="G13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H13" t="n">
         <v>3</v>
@@ -2236,7 +2350,7 @@
         <v>3</v>
       </c>
       <c r="Y13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Z13" t="n">
         <v>3</v>
@@ -2260,7 +2374,7 @@
         <v>3</v>
       </c>
       <c r="AG13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AH13" t="n">
         <v>2</v>
@@ -2296,6 +2410,15 @@
         <v>3</v>
       </c>
       <c r="AS13" t="n">
+        <v>2</v>
+      </c>
+      <c r="AT13" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU13" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV13" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2316,7 +2439,7 @@
         <v>3</v>
       </c>
       <c r="F14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G14" t="n">
         <v>1</v>
@@ -2334,7 +2457,7 @@
         <v>3</v>
       </c>
       <c r="L14" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M14" t="n">
         <v>1</v>
@@ -2373,13 +2496,13 @@
         <v>1</v>
       </c>
       <c r="Y14" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Z14" t="n">
         <v>3</v>
       </c>
       <c r="AA14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AB14" t="n">
         <v>1</v>
@@ -2400,7 +2523,7 @@
         <v>1</v>
       </c>
       <c r="AH14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AI14" t="n">
         <v>3</v>
@@ -2424,7 +2547,7 @@
         <v>3</v>
       </c>
       <c r="AP14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AQ14" t="n">
         <v>1</v>
@@ -2433,6 +2556,15 @@
         <v>3</v>
       </c>
       <c r="AS14" t="n">
+        <v>2</v>
+      </c>
+      <c r="AT14" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU14" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV14" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2459,7 +2591,7 @@
         <v>1</v>
       </c>
       <c r="H15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I15" t="n">
         <v>2</v>
@@ -2489,7 +2621,7 @@
         <v>3</v>
       </c>
       <c r="R15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S15" t="n">
         <v>2</v>
@@ -2507,7 +2639,7 @@
         <v>3</v>
       </c>
       <c r="X15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Y15" t="n">
         <v>3</v>
@@ -2522,7 +2654,7 @@
         <v>2</v>
       </c>
       <c r="AC15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AD15" t="n">
         <v>2</v>
@@ -2531,7 +2663,7 @@
         <v>1</v>
       </c>
       <c r="AF15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG15" t="n">
         <v>2</v>
@@ -2570,6 +2702,15 @@
         <v>2</v>
       </c>
       <c r="AS15" t="n">
+        <v>2</v>
+      </c>
+      <c r="AT15" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU15" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV15" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2578,7 +2719,7 @@
         <v>1</v>
       </c>
       <c r="B16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C16" t="n">
         <v>2</v>
@@ -2590,7 +2731,7 @@
         <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G16" t="n">
         <v>2</v>
@@ -2602,10 +2743,10 @@
         <v>2</v>
       </c>
       <c r="J16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L16" t="n">
         <v>2</v>
@@ -2647,13 +2788,13 @@
         <v>1</v>
       </c>
       <c r="Y16" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Z16" t="n">
         <v>3</v>
       </c>
       <c r="AA16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AB16" t="n">
         <v>1</v>
@@ -2665,7 +2806,7 @@
         <v>2</v>
       </c>
       <c r="AE16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AF16" t="n">
         <v>3</v>
@@ -2680,13 +2821,13 @@
         <v>2</v>
       </c>
       <c r="AJ16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AK16" t="n">
         <v>1</v>
       </c>
       <c r="AL16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AM16" t="n">
         <v>2</v>
@@ -2701,12 +2842,21 @@
         <v>2</v>
       </c>
       <c r="AQ16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AR16" t="n">
         <v>3</v>
       </c>
       <c r="AS16" t="n">
+        <v>2</v>
+      </c>
+      <c r="AT16" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU16" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV16" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2741,9 +2891,7 @@
       <c r="J17" t="n">
         <v>1</v>
       </c>
-      <c r="K17" t="n">
-        <v>3</v>
-      </c>
+      <c r="K17" t="inlineStr"/>
       <c r="L17" t="n">
         <v>2</v>
       </c>
@@ -2778,16 +2926,16 @@
         <v>1</v>
       </c>
       <c r="W17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="X17" t="n">
         <v>2</v>
       </c>
       <c r="Y17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Z17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AA17" t="n">
         <v>2</v>
@@ -2805,7 +2953,7 @@
         <v>1</v>
       </c>
       <c r="AF17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AG17" t="n">
         <v>2</v>
@@ -2844,6 +2992,15 @@
         <v>3</v>
       </c>
       <c r="AS17" t="n">
+        <v>2</v>
+      </c>
+      <c r="AT17" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU17" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV17" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2900,7 +3057,7 @@
         <v>3</v>
       </c>
       <c r="R18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S18" t="n">
         <v>2</v>
@@ -2921,7 +3078,7 @@
         <v>2</v>
       </c>
       <c r="Y18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Z18" t="n">
         <v>3</v>
@@ -2930,7 +3087,7 @@
         <v>2</v>
       </c>
       <c r="AB18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AC18" t="n">
         <v>3</v>
@@ -2939,13 +3096,13 @@
         <v>3</v>
       </c>
       <c r="AE18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AF18" t="n">
         <v>3</v>
       </c>
       <c r="AG18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AH18" t="n">
         <v>2</v>
@@ -2957,7 +3114,7 @@
         <v>2</v>
       </c>
       <c r="AK18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AL18" t="n">
         <v>3</v>
@@ -2966,7 +3123,7 @@
         <v>2</v>
       </c>
       <c r="AN18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AO18" t="n">
         <v>3</v>
@@ -2982,6 +3139,15 @@
       </c>
       <c r="AS18" t="n">
         <v>2</v>
+      </c>
+      <c r="AT18" t="n">
+        <v>3</v>
+      </c>
+      <c r="AU18" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV18" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="19">
@@ -3019,7 +3185,7 @@
         <v>2</v>
       </c>
       <c r="L19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M19" t="n">
         <v>1</v>
@@ -3058,13 +3224,13 @@
         <v>2</v>
       </c>
       <c r="Y19" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Z19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AA19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AB19" t="n">
         <v>1</v>
@@ -3076,13 +3242,13 @@
         <v>2</v>
       </c>
       <c r="AE19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AF19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AH19" t="n">
         <v>2</v>
@@ -3119,6 +3285,15 @@
       </c>
       <c r="AS19" t="n">
         <v>2</v>
+      </c>
+      <c r="AT19" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU19" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV19" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="20">
@@ -3201,7 +3376,7 @@
         <v>3</v>
       </c>
       <c r="AA20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AB20" t="n">
         <v>3</v>
@@ -3213,13 +3388,13 @@
         <v>2</v>
       </c>
       <c r="AE20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AF20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AG20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AH20" t="n">
         <v>3</v>
@@ -3246,7 +3421,7 @@
         <v>3</v>
       </c>
       <c r="AP20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AQ20" t="n">
         <v>3</v>
@@ -3255,6 +3430,15 @@
         <v>3</v>
       </c>
       <c r="AS20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT20" t="n">
+        <v>3</v>
+      </c>
+      <c r="AU20" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV20" t="n">
         <v>2</v>
       </c>
     </row>
@@ -3311,7 +3495,7 @@
         <v>3</v>
       </c>
       <c r="R21" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S21" t="n">
         <v>2</v>
@@ -3338,7 +3522,7 @@
         <v>3</v>
       </c>
       <c r="AA21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AB21" t="n">
         <v>2</v>
@@ -3350,22 +3534,22 @@
         <v>2</v>
       </c>
       <c r="AE21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AF21" t="n">
         <v>3</v>
       </c>
       <c r="AG21" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AH21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AI21" t="n">
         <v>3</v>
       </c>
       <c r="AJ21" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AK21" t="n">
         <v>2</v>
@@ -3392,6 +3576,15 @@
         <v>3</v>
       </c>
       <c r="AS21" t="n">
+        <v>2</v>
+      </c>
+      <c r="AT21" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU21" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV21" t="n">
         <v>2</v>
       </c>
     </row>
@@ -3418,25 +3611,25 @@
         <v>1</v>
       </c>
       <c r="H22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J22" t="n">
         <v>1</v>
       </c>
       <c r="K22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L22" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M22" t="n">
         <v>1</v>
       </c>
       <c r="N22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O22" t="n">
         <v>1</v>
@@ -3448,7 +3641,7 @@
         <v>2</v>
       </c>
       <c r="R22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S22" t="n">
         <v>1</v>
@@ -3466,16 +3659,16 @@
         <v>1</v>
       </c>
       <c r="X22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Y22" t="n">
         <v>3</v>
       </c>
       <c r="Z22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AA22" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AB22" t="n">
         <v>1</v>
@@ -3487,10 +3680,10 @@
         <v>2</v>
       </c>
       <c r="AE22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AF22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG22" t="n">
         <v>2</v>
@@ -3517,7 +3710,7 @@
         <v>1</v>
       </c>
       <c r="AO22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AP22" t="n">
         <v>2</v>
@@ -3529,6 +3722,15 @@
         <v>2</v>
       </c>
       <c r="AS22" t="n">
+        <v>2</v>
+      </c>
+      <c r="AT22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU22" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV22" t="n">
         <v>2</v>
       </c>
     </row>
@@ -3552,7 +3754,7 @@
         <v>2</v>
       </c>
       <c r="G23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H23" t="n">
         <v>2</v>
@@ -3600,16 +3802,16 @@
         <v>1</v>
       </c>
       <c r="W23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="X23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Y23" t="n">
         <v>3</v>
       </c>
       <c r="Z23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AA23" t="n">
         <v>2</v>
@@ -3666,6 +3868,15 @@
         <v>2</v>
       </c>
       <c r="AS23" t="n">
+        <v>2</v>
+      </c>
+      <c r="AT23" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU23" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV23" t="n">
         <v>2</v>
       </c>
     </row>
@@ -3674,7 +3885,7 @@
         <v>1</v>
       </c>
       <c r="B24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C24" t="n">
         <v>2</v>
@@ -3689,7 +3900,7 @@
         <v>2</v>
       </c>
       <c r="G24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H24" t="n">
         <v>2</v>
@@ -3743,16 +3954,16 @@
         <v>2</v>
       </c>
       <c r="Y24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Z24" t="n">
         <v>3</v>
       </c>
       <c r="AA24" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AB24" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AC24" t="n">
         <v>3</v>
@@ -3767,7 +3978,7 @@
         <v>3</v>
       </c>
       <c r="AG24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AH24" t="n">
         <v>2</v>
@@ -3791,7 +4002,7 @@
         <v>1</v>
       </c>
       <c r="AO24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AP24" t="n">
         <v>2</v>
@@ -3803,6 +4014,15 @@
         <v>3</v>
       </c>
       <c r="AS24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AT24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AU24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV24" t="n">
         <v>2</v>
       </c>
     </row>
@@ -3817,7 +4037,7 @@
         <v>1</v>
       </c>
       <c r="D25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E25" t="n">
         <v>2</v>
@@ -3834,12 +4054,8 @@
       <c r="I25" t="n">
         <v>1</v>
       </c>
-      <c r="J25" t="n">
-        <v>2</v>
-      </c>
-      <c r="K25" t="n">
-        <v>2</v>
-      </c>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
       <c r="L25" t="n">
         <v>1</v>
       </c>
@@ -3847,14 +4063,12 @@
         <v>2</v>
       </c>
       <c r="N25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O25" t="n">
         <v>1</v>
       </c>
-      <c r="P25" t="n">
-        <v>2</v>
-      </c>
+      <c r="P25" t="inlineStr"/>
       <c r="Q25" t="n">
         <v>2</v>
       </c>
@@ -3883,16 +4097,16 @@
         <v>2</v>
       </c>
       <c r="Z25" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AA25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AB25" t="n">
         <v>2</v>
       </c>
       <c r="AC25" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AD25" t="n">
         <v>1</v>
@@ -3901,7 +4115,7 @@
         <v>1</v>
       </c>
       <c r="AF25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AG25" t="n">
         <v>1</v>
@@ -3919,7 +4133,7 @@
         <v>2</v>
       </c>
       <c r="AL25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AM25" t="n">
         <v>1</v>
@@ -3940,6 +4154,15 @@
         <v>2</v>
       </c>
       <c r="AS25" t="n">
+        <v>2</v>
+      </c>
+      <c r="AT25" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU25" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV25" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3969,7 +4192,7 @@
         <v>3</v>
       </c>
       <c r="I26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J26" t="n">
         <v>2</v>
@@ -4017,13 +4240,13 @@
         <v>3</v>
       </c>
       <c r="Y26" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Z26" t="n">
         <v>3</v>
       </c>
       <c r="AA26" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AB26" t="n">
         <v>2</v>
@@ -4035,7 +4258,7 @@
         <v>2</v>
       </c>
       <c r="AE26" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AF26" t="n">
         <v>3</v>
@@ -4044,7 +4267,7 @@
         <v>2</v>
       </c>
       <c r="AH26" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AI26" t="n">
         <v>3</v>
@@ -4077,12 +4300,21 @@
         <v>3</v>
       </c>
       <c r="AS26" t="n">
+        <v>2</v>
+      </c>
+      <c r="AT26" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV26" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B27" t="n">
         <v>1</v>
@@ -4127,7 +4359,7 @@
         <v>2</v>
       </c>
       <c r="P27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q27" t="n">
         <v>1</v>
@@ -4145,7 +4377,7 @@
         <v>2</v>
       </c>
       <c r="V27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W27" t="n">
         <v>1</v>
@@ -4154,13 +4386,13 @@
         <v>2</v>
       </c>
       <c r="Y27" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Z27" t="n">
         <v>3</v>
       </c>
       <c r="AA27" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AB27" t="n">
         <v>1</v>
@@ -4184,7 +4416,7 @@
         <v>2</v>
       </c>
       <c r="AI27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AJ27" t="n">
         <v>2</v>
@@ -4208,12 +4440,21 @@
         <v>2</v>
       </c>
       <c r="AQ27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AR27" t="n">
         <v>1</v>
       </c>
       <c r="AS27" t="n">
+        <v>2</v>
+      </c>
+      <c r="AT27" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU27" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV27" t="n">
         <v>2</v>
       </c>
     </row>
@@ -4291,7 +4532,7 @@
         <v>2</v>
       </c>
       <c r="Y28" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Z28" t="n">
         <v>3</v>
@@ -4309,7 +4550,7 @@
         <v>2</v>
       </c>
       <c r="AE28" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AF28" t="n">
         <v>3</v>
@@ -4351,6 +4592,15 @@
         <v>3</v>
       </c>
       <c r="AS28" t="n">
+        <v>2</v>
+      </c>
+      <c r="AT28" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU28" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV28" t="n">
         <v>2</v>
       </c>
     </row>
@@ -4382,9 +4632,7 @@
       <c r="I29" t="n">
         <v>1</v>
       </c>
-      <c r="J29" t="n">
-        <v>1</v>
-      </c>
+      <c r="J29" t="inlineStr"/>
       <c r="K29" t="n">
         <v>2</v>
       </c>
@@ -4431,10 +4679,10 @@
         <v>1</v>
       </c>
       <c r="Z29" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AA29" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AB29" t="n">
         <v>1</v>
@@ -4443,7 +4691,7 @@
         <v>2</v>
       </c>
       <c r="AD29" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AE29" t="n">
         <v>1</v>
@@ -4455,7 +4703,7 @@
         <v>1</v>
       </c>
       <c r="AH29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AI29" t="n">
         <v>2</v>
@@ -4488,6 +4736,15 @@
         <v>2</v>
       </c>
       <c r="AS29" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT29" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU29" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV29" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4502,13 +4759,13 @@
         <v>1</v>
       </c>
       <c r="D30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E30" t="n">
         <v>2</v>
       </c>
       <c r="F30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G30" t="n">
         <v>1</v>
@@ -4565,10 +4822,10 @@
         <v>1</v>
       </c>
       <c r="Y30" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Z30" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AA30" t="n">
         <v>3</v>
@@ -4586,7 +4843,7 @@
         <v>1</v>
       </c>
       <c r="AF30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AG30" t="n">
         <v>1</v>
@@ -4625,6 +4882,15 @@
         <v>2</v>
       </c>
       <c r="AS30" t="n">
+        <v>2</v>
+      </c>
+      <c r="AT30" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU30" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV30" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4762,6 +5028,15 @@
         <v>3</v>
       </c>
       <c r="AS31" t="n">
+        <v>3</v>
+      </c>
+      <c r="AT31" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU31" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV31" t="n">
         <v>3</v>
       </c>
     </row>

</xml_diff>